<commit_message>
Open submission workbook on task list sheet
</commit_message>
<xml_diff>
--- a/Nhom1_CS13.xlsx
+++ b/Nhom1_CS13.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\K4-L3-CS13-NaCl-AI-Roadmap\mydocs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\K4-L3-CS13-NaCl-AI-Roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F68988B4-1F4A-4D97-B438-500F342231F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="0_Hướng dẫn" sheetId="1" r:id="rId1"/>

</xml_diff>